<commit_message>
Complete Accounts test execution and reporting
</commit_message>
<xml_diff>
--- a/04-RTM/Accounts-RTM-v1.0.xlsx
+++ b/04-RTM/Accounts-RTM-v1.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SIDDIQ\EspoCRM-QA-Automation\04-RTM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{273ED156-9B94-444B-89FA-0C05031175DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3D1486F-7F30-4812-B6D7-8D5190A6CC64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="75">
   <si>
     <t>Requirement ID</t>
   </si>
@@ -109,6 +109,147 @@
   </si>
   <si>
     <t>TC-ACC-011</t>
+  </si>
+  <si>
+    <t>FR-ACC-017</t>
+  </si>
+  <si>
+    <t>TS-ACC-017</t>
+  </si>
+  <si>
+    <t>TC-ACC-012</t>
+  </si>
+  <si>
+    <t>FR-ACC-018</t>
+  </si>
+  <si>
+    <t>TS-ACC-018</t>
+  </si>
+  <si>
+    <t>TC-ACC-013</t>
+  </si>
+  <si>
+    <t>TC-ACC-014</t>
+  </si>
+  <si>
+    <t>FR-ACC-019</t>
+  </si>
+  <si>
+    <t>TS-ACC-019</t>
+  </si>
+  <si>
+    <t>TC-ACC-015</t>
+  </si>
+  <si>
+    <t>TC-ACC-016</t>
+  </si>
+  <si>
+    <t>TC-ACC-017</t>
+  </si>
+  <si>
+    <t>FR-ACC-020</t>
+  </si>
+  <si>
+    <t>TS-ACC-020</t>
+  </si>
+  <si>
+    <t>TC-ACC-018</t>
+  </si>
+  <si>
+    <t>TC-ACC-019</t>
+  </si>
+  <si>
+    <t>FR-ACC-021</t>
+  </si>
+  <si>
+    <t>TS-ACC-021</t>
+  </si>
+  <si>
+    <t>TC-ACC-020</t>
+  </si>
+  <si>
+    <t>FR-ACC-022</t>
+  </si>
+  <si>
+    <t>TS-ACC-022</t>
+  </si>
+  <si>
+    <t>TC-ACC-021</t>
+  </si>
+  <si>
+    <t>TC-ACC-022</t>
+  </si>
+  <si>
+    <t>TC-ACC-023</t>
+  </si>
+  <si>
+    <t>TC-ACC-024</t>
+  </si>
+  <si>
+    <t>FR-ACC-023</t>
+  </si>
+  <si>
+    <t>TS-ACC-023</t>
+  </si>
+  <si>
+    <t>TC-ACC-025</t>
+  </si>
+  <si>
+    <t>FR-ACC-024</t>
+  </si>
+  <si>
+    <t>TS-ACC-024</t>
+  </si>
+  <si>
+    <t>TC-ACC-026</t>
+  </si>
+  <si>
+    <t>FR-ACC-025</t>
+  </si>
+  <si>
+    <t>TS-ACC-025</t>
+  </si>
+  <si>
+    <t>TC-ACC-027</t>
+  </si>
+  <si>
+    <t>TC-ACC-028</t>
+  </si>
+  <si>
+    <t>TC-ACC-029</t>
+  </si>
+  <si>
+    <t>FR-ACC-013</t>
+  </si>
+  <si>
+    <t>TS-ACC-013</t>
+  </si>
+  <si>
+    <t>TC-ACC-030</t>
+  </si>
+  <si>
+    <t>TC-ACC-031</t>
+  </si>
+  <si>
+    <t>FR-ACC-016</t>
+  </si>
+  <si>
+    <t>TS-ACC-016</t>
+  </si>
+  <si>
+    <t>TC-ACC-032</t>
+  </si>
+  <si>
+    <t>TC-ACC-033</t>
+  </si>
+  <si>
+    <t>TC-ACC-034</t>
+  </si>
+  <si>
+    <t>TC-ACC-035</t>
+  </si>
+  <si>
+    <t>TC-ACC-036</t>
   </si>
 </sst>
 </file>
@@ -167,13 +308,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -455,7 +599,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.21875" bestFit="1" customWidth="1"/>
@@ -632,6 +776,356 @@
         <v>7</v>
       </c>
     </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A32" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A33" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A34" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A35" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A36" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A37" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>